<commit_message>
Libro combinado V1.3: combinar_libros.py, corrección de referencias de fila y fila Formulario F
- scripts/combinar_libros.py: copia solo celdas de entrada de Participantes y Respuestas editando el XML; no sobrescribe, no modifica base ni fuente.
- scripts/libro_xml.py: desplaza filas cambiando TODAS las referencias relativas y verifica que cada fórmula apunte a su fila (causa del error de la columna K de P26-P28). Generador del libro V1.3 corregido; Resumen con Formulario F; libro vacío regenerado.
- Libro real combinado y su ingesta: fuera de Git (28 participantes, 181 frases, 169 decisiones sin cambios). Solo cifras en el registro.
- Pruebas: transcripción 42/42, conciliación 28/28, compuertas 67/67, piloto 51/51, lote real 78/78; verificar_referencias 0 discrepancias.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/lote_real_1/Lote1_Transcripcion_V1.3.xlsx
+++ b/docs/lote_real_1/Lote1_Transcripcion_V1.3.xlsx
@@ -2473,7 +2473,7 @@
         <v>0</v>
       </c>
       <c r="K29" s="8" t="str">
-        <f aca="false">IF(C29="Transcrito",I28-J29,"")</f>
+        <f aca="false">IF(C29="Transcrito",I29-J29,"")</f>
         <v/>
       </c>
       <c r="L29" s="9" t="str">
@@ -2510,7 +2510,7 @@
         <v>0</v>
       </c>
       <c r="K30" s="8" t="str">
-        <f aca="false">IF(C30="Transcrito",I28-J30,"")</f>
+        <f aca="false">IF(C30="Transcrito",I30-J30,"")</f>
         <v/>
       </c>
       <c r="L30" s="9" t="str">
@@ -2547,7 +2547,7 @@
         <v>0</v>
       </c>
       <c r="K31" s="8" t="str">
-        <f aca="false">IF(C31="Transcrito",I28-J31,"")</f>
+        <f aca="false">IF(C31="Transcrito",I31-J31,"")</f>
         <v/>
       </c>
       <c r="L31" s="9" t="str">
@@ -10328,7 +10328,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
@@ -10553,6 +10553,19 @@
       </c>
       <c r="C28" s="18" t="str">
         <f aca="false">"Aplicados sin transcribir: "&amp;COUNTIFS(Participantes!$B$4:$B$31,"E",Participantes!$C$4:$C$31,"Aplicado")</f>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Formulario F</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="n">
+        <f aca="false">COUNTIFS(Participantes!$B$4:$B$31,"F",Participantes!$C$4:$C$31,"Transcrito")</f>
+      </c>
+      <c r="C29" s="18" t="str">
+        <f aca="false">"Aplicados sin transcribir: "&amp;COUNTIFS(Participantes!$B$4:$B$31,"F",Participantes!$C$4:$C$31,"Aplicado")</f>
       </c>
     </row>
   </sheetData>

</xml_diff>